<commit_message>
Update agreement, office sheet, 211 sheet, tracker; add PFA and NLG logos
</commit_message>
<xml_diff>
--- a/assets/SSA-Signup-Prescreen-Tracker.xlsx
+++ b/assets/SSA-Signup-Prescreen-Tracker.xlsx
@@ -3806,7 +3806,7 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>5. Social Security Administration only: do the prescreen FIRST (Child questions, or 18 Plus questions) to see if they qualify to apply.</t>
+          <t>5. Social Security Administration only: do the prescreen FIRST (Child questions, or 18 Plus questions) to see if they qualify to apply. Guidance includes 2 free 30-minute sessions; further assistance or guidance is $10.00 for every 30 minutes needed.</t>
         </is>
       </c>
     </row>
@@ -3834,7 +3834,7 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>9. MEDICATION ASSISTANCE: also check if we are able to assist on any of our programs (Texas Care Rx, manufacturer assistance programs, GoodRx, Cost Plus Drugs). Record it on the Medication Assistance sheet. The client will receive an email with the result.</t>
+          <t>9. MEDICATION ASSISTANCE: also check if we are able to assist on any of our programs (Texas Care Rx, manufacturer assistance programs, GoodRx, Cost Plus Drugs). Record it on the Medication Assistance sheet. The client will receive an email with the result and the information. If the client needs assistance to fill out the application, a donation is requested.</t>
         </is>
       </c>
     </row>

</xml_diff>